<commit_message>
chore: actualización automática 2026-07-15
</commit_message>
<xml_diff>
--- a/Base_Andina_Ventas_Auto.xlsx
+++ b/Base_Andina_Ventas_Auto.xlsx
@@ -17384,7 +17384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G401"/>
+  <dimension ref="A1:G426"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -28969,6 +28969,727 @@
         <v>826</v>
       </c>
     </row>
+    <row r="402">
+      <c r="A402" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B402" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C402" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D402" s="2" t="inlineStr">
+        <is>
+          <t>Changan</t>
+        </is>
+      </c>
+      <c r="E402" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F402" s="2" t="n">
+        <v>7430</v>
+      </c>
+      <c r="G402" s="2" t="n">
+        <v>1309</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B403" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C403" t="n">
+        <v>6</v>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Chery</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F403" t="n">
+        <v>4264</v>
+      </c>
+      <c r="G403" t="n">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B404" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C404" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D404" s="2" t="inlineStr">
+        <is>
+          <t>Chevrolet</t>
+        </is>
+      </c>
+      <c r="E404" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F404" s="2" t="n">
+        <v>8226</v>
+      </c>
+      <c r="G404" s="2" t="n">
+        <v>1409</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B405" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C405" t="n">
+        <v>6</v>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Citroen</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F405" t="n">
+        <v>2121</v>
+      </c>
+      <c r="G405" t="n">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B406" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C406" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D406" s="2" t="inlineStr">
+        <is>
+          <t>Ford</t>
+        </is>
+      </c>
+      <c r="E406" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F406" s="2" t="n">
+        <v>7842</v>
+      </c>
+      <c r="G406" s="2" t="n">
+        <v>1467</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B407" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C407" t="n">
+        <v>6</v>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Foton</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F407" t="n">
+        <v>3198</v>
+      </c>
+      <c r="G407" t="n">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B408" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C408" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D408" s="2" t="inlineStr">
+        <is>
+          <t>Geely</t>
+        </is>
+      </c>
+      <c r="E408" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F408" s="2" t="n">
+        <v>2978</v>
+      </c>
+      <c r="G408" s="2" t="n">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B409" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C409" t="n">
+        <v>6</v>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>Great Wall</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F409" t="n">
+        <v>8034</v>
+      </c>
+      <c r="G409" t="n">
+        <v>1227</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B410" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C410" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D410" s="2" t="inlineStr">
+        <is>
+          <t>Hyundai</t>
+        </is>
+      </c>
+      <c r="E410" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F410" s="2" t="n">
+        <v>10062</v>
+      </c>
+      <c r="G410" s="2" t="n">
+        <v>1722</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B411" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C411" t="n">
+        <v>6</v>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Jac</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F411" t="n">
+        <v>3293</v>
+      </c>
+      <c r="G411" t="n">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B412" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C412" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D412" s="2" t="inlineStr">
+        <is>
+          <t>Jeep</t>
+        </is>
+      </c>
+      <c r="E412" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F412" s="2" t="n">
+        <v>1721</v>
+      </c>
+      <c r="G412" s="2" t="inlineStr"/>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B413" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C413" t="n">
+        <v>6</v>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Jetour</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F413" t="n">
+        <v>3670</v>
+      </c>
+      <c r="G413" t="n">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B414" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C414" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D414" s="2" t="inlineStr">
+        <is>
+          <t>Kia</t>
+        </is>
+      </c>
+      <c r="E414" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F414" s="2" t="n">
+        <v>8995</v>
+      </c>
+      <c r="G414" s="2" t="n">
+        <v>1420</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B415" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C415" t="n">
+        <v>6</v>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Maxus</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F415" t="n">
+        <v>3002</v>
+      </c>
+      <c r="G415" t="n">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B416" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C416" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D416" s="2" t="inlineStr">
+        <is>
+          <t>Mazda</t>
+        </is>
+      </c>
+      <c r="E416" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F416" s="2" t="n">
+        <v>4592</v>
+      </c>
+      <c r="G416" s="2" t="n">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B417" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C417" t="n">
+        <v>6</v>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Mg</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F417" t="n">
+        <v>5708</v>
+      </c>
+      <c r="G417" t="n">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B418" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C418" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D418" s="2" t="inlineStr">
+        <is>
+          <t>Mitsubishi</t>
+        </is>
+      </c>
+      <c r="E418" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F418" s="2" t="n">
+        <v>5911</v>
+      </c>
+      <c r="G418" s="2" t="n">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B419" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C419" t="n">
+        <v>6</v>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Omoda</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F419" t="n">
+        <v>2610</v>
+      </c>
+      <c r="G419" t="n">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B420" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C420" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D420" s="2" t="inlineStr">
+        <is>
+          <t>Peugeot</t>
+        </is>
+      </c>
+      <c r="E420" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F420" s="2" t="n">
+        <v>6834</v>
+      </c>
+      <c r="G420" s="2" t="n">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B421" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C421" t="n">
+        <v>6</v>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Ram</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F421" t="n">
+        <v>2210</v>
+      </c>
+      <c r="G421" t="n">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B422" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C422" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D422" s="2" t="inlineStr">
+        <is>
+          <t>Subaru</t>
+        </is>
+      </c>
+      <c r="E422" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F422" s="2" t="n">
+        <v>3035</v>
+      </c>
+      <c r="G422" s="2" t="n">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B423" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C423" t="n">
+        <v>6</v>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F423" t="n">
+        <v>11782</v>
+      </c>
+      <c r="G423" t="n">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B424" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C424" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D424" s="2" t="inlineStr">
+        <is>
+          <t>Tesla</t>
+        </is>
+      </c>
+      <c r="E424" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F424" s="2" t="n">
+        <v>1687</v>
+      </c>
+      <c r="G424" s="2" t="inlineStr"/>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B425" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C425" t="n">
+        <v>6</v>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F425" t="n">
+        <v>12657</v>
+      </c>
+      <c r="G425" t="n">
+        <v>2160</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B426" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C426" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D426" s="2" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="E426" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F426" s="2" t="n">
+        <v>3637</v>
+      </c>
+      <c r="G426" s="2" t="n">
+        <v>468</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -28980,7 +29701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G504"/>
+  <dimension ref="A1:G584"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -43322,6 +44043,2322 @@
       </c>
       <c r="G504" s="2" t="n">
         <v>266</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B505" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C505" t="n">
+        <v>2</v>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>Byd</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F505" t="n">
+        <v>699</v>
+      </c>
+      <c r="G505" t="n">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B506" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C506" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D506" s="2" t="inlineStr">
+        <is>
+          <t>Changan</t>
+        </is>
+      </c>
+      <c r="E506" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F506" s="2" t="n">
+        <v>367</v>
+      </c>
+      <c r="G506" s="2" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B507" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C507" t="n">
+        <v>2</v>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>Chery</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F507" t="n">
+        <v>1189</v>
+      </c>
+      <c r="G507" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B508" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C508" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D508" s="2" t="inlineStr">
+        <is>
+          <t>Chevrolet</t>
+        </is>
+      </c>
+      <c r="E508" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F508" s="2" t="n">
+        <v>2802</v>
+      </c>
+      <c r="G508" s="2" t="n">
+        <v>1317</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B509" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C509" t="n">
+        <v>2</v>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>Dfsk</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F509" t="n">
+        <v>592</v>
+      </c>
+      <c r="G509" t="n">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B510" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C510" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D510" s="2" t="inlineStr">
+        <is>
+          <t>Dongfeng</t>
+        </is>
+      </c>
+      <c r="E510" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F510" s="2" t="n">
+        <v>762</v>
+      </c>
+      <c r="G510" s="2" t="n">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B511" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C511" t="n">
+        <v>2</v>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Ford</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F511" t="n">
+        <v>308</v>
+      </c>
+      <c r="G511" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B512" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C512" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D512" s="2" t="inlineStr">
+        <is>
+          <t>Foton</t>
+        </is>
+      </c>
+      <c r="E512" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F512" s="2" t="n">
+        <v>364</v>
+      </c>
+      <c r="G512" s="2" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B513" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C513" t="n">
+        <v>2</v>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Gwm</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F513" t="n">
+        <v>1229</v>
+      </c>
+      <c r="G513" t="n">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B514" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C514" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D514" s="2" t="inlineStr">
+        <is>
+          <t>Hino</t>
+        </is>
+      </c>
+      <c r="E514" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F514" s="2" t="n">
+        <v>331</v>
+      </c>
+      <c r="G514" s="2" t="n">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B515" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C515" t="n">
+        <v>2</v>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Hyundai</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F515" t="n">
+        <v>1330</v>
+      </c>
+      <c r="G515" t="n">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B516" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C516" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D516" s="2" t="inlineStr">
+        <is>
+          <t>Jac</t>
+        </is>
+      </c>
+      <c r="E516" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F516" s="2" t="n">
+        <v>772</v>
+      </c>
+      <c r="G516" s="2" t="n">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B517" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C517" t="n">
+        <v>2</v>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Jetour</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F517" t="n">
+        <v>503</v>
+      </c>
+      <c r="G517" t="n">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B518" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C518" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D518" s="2" t="inlineStr">
+        <is>
+          <t>Kia</t>
+        </is>
+      </c>
+      <c r="E518" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F518" s="2" t="n">
+        <v>3525</v>
+      </c>
+      <c r="G518" s="2" t="n">
+        <v>1770</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B519" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C519" t="n">
+        <v>2</v>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>Mazda</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F519" t="n">
+        <v>588</v>
+      </c>
+      <c r="G519" t="n">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B520" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C520" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D520" s="2" t="inlineStr">
+        <is>
+          <t>Renault</t>
+        </is>
+      </c>
+      <c r="E520" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F520" s="2" t="n">
+        <v>589</v>
+      </c>
+      <c r="G520" s="2" t="n">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B521" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C521" t="n">
+        <v>2</v>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Sinotruk</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F521" t="n">
+        <v>674</v>
+      </c>
+      <c r="G521" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B522" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C522" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D522" s="2" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="E522" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F522" s="2" t="n">
+        <v>640</v>
+      </c>
+      <c r="G522" s="2" t="n">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B523" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C523" t="n">
+        <v>2</v>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F523" t="n">
+        <v>1069</v>
+      </c>
+      <c r="G523" t="n">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B524" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C524" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D524" s="2" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="E524" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F524" s="2" t="n">
+        <v>428</v>
+      </c>
+      <c r="G524" s="2" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B525" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C525" t="n">
+        <v>3</v>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>Byd</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F525" t="n">
+        <v>1160</v>
+      </c>
+      <c r="G525" t="n">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B526" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C526" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D526" s="2" t="inlineStr">
+        <is>
+          <t>Changan</t>
+        </is>
+      </c>
+      <c r="E526" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F526" s="2" t="n">
+        <v>684</v>
+      </c>
+      <c r="G526" s="2" t="n">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B527" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C527" t="n">
+        <v>3</v>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>Chery</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F527" t="n">
+        <v>1851</v>
+      </c>
+      <c r="G527" t="n">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B528" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C528" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D528" s="2" t="inlineStr">
+        <is>
+          <t>Chevrolet</t>
+        </is>
+      </c>
+      <c r="E528" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F528" s="2" t="n">
+        <v>4181</v>
+      </c>
+      <c r="G528" s="2" t="n">
+        <v>1379</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B529" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C529" t="n">
+        <v>3</v>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>Dfsk</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F529" t="n">
+        <v>1009</v>
+      </c>
+      <c r="G529" t="n">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B530" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C530" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D530" s="2" t="inlineStr">
+        <is>
+          <t>Dongfeng</t>
+        </is>
+      </c>
+      <c r="E530" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F530" s="2" t="n">
+        <v>1256</v>
+      </c>
+      <c r="G530" s="2" t="n">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B531" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C531" t="n">
+        <v>3</v>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>Ford</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F531" t="n">
+        <v>530</v>
+      </c>
+      <c r="G531" t="n">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B532" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C532" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D532" s="2" t="inlineStr">
+        <is>
+          <t>Foton</t>
+        </is>
+      </c>
+      <c r="E532" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F532" s="2" t="n">
+        <v>610</v>
+      </c>
+      <c r="G532" s="2" t="n">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B533" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C533" t="n">
+        <v>3</v>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>Gwm</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F533" t="n">
+        <v>2126</v>
+      </c>
+      <c r="G533" t="n">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B534" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C534" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D534" s="2" t="inlineStr">
+        <is>
+          <t>Hino</t>
+        </is>
+      </c>
+      <c r="E534" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F534" s="2" t="n">
+        <v>504</v>
+      </c>
+      <c r="G534" s="2" t="n">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B535" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C535" t="n">
+        <v>3</v>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>Hyundai</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F535" t="n">
+        <v>2092</v>
+      </c>
+      <c r="G535" t="n">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B536" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C536" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D536" s="2" t="inlineStr">
+        <is>
+          <t>Jac</t>
+        </is>
+      </c>
+      <c r="E536" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F536" s="2" t="n">
+        <v>1268</v>
+      </c>
+      <c r="G536" s="2" t="n">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B537" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C537" t="n">
+        <v>3</v>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>Jetour</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F537" t="n">
+        <v>838</v>
+      </c>
+      <c r="G537" t="n">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B538" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C538" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D538" s="2" t="inlineStr">
+        <is>
+          <t>Kia</t>
+        </is>
+      </c>
+      <c r="E538" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F538" s="2" t="n">
+        <v>5735</v>
+      </c>
+      <c r="G538" s="2" t="n">
+        <v>2210</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B539" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C539" t="n">
+        <v>3</v>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>Mazda</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F539" t="n">
+        <v>876</v>
+      </c>
+      <c r="G539" t="n">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B540" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C540" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D540" s="2" t="inlineStr">
+        <is>
+          <t>Renault</t>
+        </is>
+      </c>
+      <c r="E540" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F540" s="2" t="n">
+        <v>845</v>
+      </c>
+      <c r="G540" s="2" t="n">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B541" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C541" t="n">
+        <v>3</v>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>Sinotruk</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F541" t="n">
+        <v>1092</v>
+      </c>
+      <c r="G541" t="n">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B542" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C542" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D542" s="2" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="E542" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F542" s="2" t="n">
+        <v>1150</v>
+      </c>
+      <c r="G542" s="2" t="n">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B543" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C543" t="n">
+        <v>3</v>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F543" t="n">
+        <v>1741</v>
+      </c>
+      <c r="G543" t="n">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B544" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C544" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D544" s="2" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="E544" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F544" s="2" t="n">
+        <v>745</v>
+      </c>
+      <c r="G544" s="2" t="n">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B545" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C545" t="n">
+        <v>4</v>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>Byd</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F545" t="n">
+        <v>1510</v>
+      </c>
+      <c r="G545" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B546" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C546" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D546" s="2" t="inlineStr">
+        <is>
+          <t>Changan</t>
+        </is>
+      </c>
+      <c r="E546" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F546" s="2" t="n">
+        <v>911</v>
+      </c>
+      <c r="G546" s="2" t="n">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B547" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C547" t="n">
+        <v>4</v>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Chery</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F547" t="n">
+        <v>2505</v>
+      </c>
+      <c r="G547" t="n">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B548" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C548" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D548" s="2" t="inlineStr">
+        <is>
+          <t>Chevrolet</t>
+        </is>
+      </c>
+      <c r="E548" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F548" s="2" t="n">
+        <v>6118</v>
+      </c>
+      <c r="G548" s="2" t="n">
+        <v>1937</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B549" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C549" t="n">
+        <v>4</v>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>Dfsk</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F549" t="n">
+        <v>1394</v>
+      </c>
+      <c r="G549" t="n">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B550" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C550" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D550" s="2" t="inlineStr">
+        <is>
+          <t>Dongfeng</t>
+        </is>
+      </c>
+      <c r="E550" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F550" s="2" t="n">
+        <v>1790</v>
+      </c>
+      <c r="G550" s="2" t="n">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B551" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C551" t="n">
+        <v>4</v>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>Ford</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F551" t="n">
+        <v>690</v>
+      </c>
+      <c r="G551" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B552" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C552" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D552" s="2" t="inlineStr">
+        <is>
+          <t>Foton</t>
+        </is>
+      </c>
+      <c r="E552" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F552" s="2" t="n">
+        <v>853</v>
+      </c>
+      <c r="G552" s="2" t="n">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B553" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C553" t="n">
+        <v>4</v>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>Gwm</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F553" t="n">
+        <v>2790</v>
+      </c>
+      <c r="G553" t="n">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B554" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C554" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D554" s="2" t="inlineStr">
+        <is>
+          <t>Hyundai</t>
+        </is>
+      </c>
+      <c r="E554" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F554" s="2" t="n">
+        <v>2888</v>
+      </c>
+      <c r="G554" s="2" t="n">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B555" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C555" t="n">
+        <v>4</v>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>Isuzu</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F555" t="n">
+        <v>692</v>
+      </c>
+      <c r="G555" t="inlineStr"/>
+    </row>
+    <row r="556">
+      <c r="A556" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B556" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C556" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D556" s="2" t="inlineStr">
+        <is>
+          <t>Jac</t>
+        </is>
+      </c>
+      <c r="E556" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F556" s="2" t="n">
+        <v>1783</v>
+      </c>
+      <c r="G556" s="2" t="n">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B557" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C557" t="n">
+        <v>4</v>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>Jetour</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F557" t="n">
+        <v>1197</v>
+      </c>
+      <c r="G557" t="n">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B558" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C558" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D558" s="2" t="inlineStr">
+        <is>
+          <t>Kia</t>
+        </is>
+      </c>
+      <c r="E558" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F558" s="2" t="n">
+        <v>8052</v>
+      </c>
+      <c r="G558" s="2" t="n">
+        <v>2317</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B559" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C559" t="n">
+        <v>4</v>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>Mazda</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F559" t="n">
+        <v>1144</v>
+      </c>
+      <c r="G559" t="n">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B560" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C560" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D560" s="2" t="inlineStr">
+        <is>
+          <t>Renault</t>
+        </is>
+      </c>
+      <c r="E560" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F560" s="2" t="n">
+        <v>962</v>
+      </c>
+      <c r="G560" s="2" t="n">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B561" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C561" t="n">
+        <v>4</v>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>Sinotruk</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F561" t="n">
+        <v>1628</v>
+      </c>
+      <c r="G561" t="n">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B562" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C562" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D562" s="2" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="E562" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F562" s="2" t="n">
+        <v>1583</v>
+      </c>
+      <c r="G562" s="2" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B563" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C563" t="n">
+        <v>4</v>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F563" t="n">
+        <v>2436</v>
+      </c>
+      <c r="G563" t="n">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B564" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C564" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D564" s="2" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="E564" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F564" s="2" t="n">
+        <v>1098</v>
+      </c>
+      <c r="G564" s="2" t="n">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B565" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C565" t="n">
+        <v>5</v>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>Byd</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F565" t="n">
+        <v>1776</v>
+      </c>
+      <c r="G565" t="n">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B566" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C566" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D566" s="2" t="inlineStr">
+        <is>
+          <t>Changan</t>
+        </is>
+      </c>
+      <c r="E566" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F566" s="2" t="n">
+        <v>1161</v>
+      </c>
+      <c r="G566" s="2" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B567" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C567" t="n">
+        <v>5</v>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>Chery</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F567" t="n">
+        <v>3142</v>
+      </c>
+      <c r="G567" t="n">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B568" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C568" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D568" s="2" t="inlineStr">
+        <is>
+          <t>Chevrolet</t>
+        </is>
+      </c>
+      <c r="E568" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F568" s="2" t="n">
+        <v>7732</v>
+      </c>
+      <c r="G568" s="2" t="n">
+        <v>1614</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B569" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C569" t="n">
+        <v>5</v>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>Dfsk</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F569" t="n">
+        <v>1832</v>
+      </c>
+      <c r="G569" t="n">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B570" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C570" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D570" s="2" t="inlineStr">
+        <is>
+          <t>Dongfeng</t>
+        </is>
+      </c>
+      <c r="E570" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F570" s="2" t="n">
+        <v>2247</v>
+      </c>
+      <c r="G570" s="2" t="n">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B571" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C571" t="n">
+        <v>5</v>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>Ford</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F571" t="n">
+        <v>814</v>
+      </c>
+      <c r="G571" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B572" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C572" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D572" s="2" t="inlineStr">
+        <is>
+          <t>Foton</t>
+        </is>
+      </c>
+      <c r="E572" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F572" s="2" t="n">
+        <v>1110</v>
+      </c>
+      <c r="G572" s="2" t="n">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B573" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C573" t="n">
+        <v>5</v>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>Gwm</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F573" t="n">
+        <v>3508</v>
+      </c>
+      <c r="G573" t="n">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B574" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C574" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D574" s="2" t="inlineStr">
+        <is>
+          <t>Hino</t>
+        </is>
+      </c>
+      <c r="E574" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F574" s="2" t="n">
+        <v>865</v>
+      </c>
+      <c r="G574" s="2" t="inlineStr"/>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B575" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C575" t="n">
+        <v>5</v>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>Hyundai</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F575" t="n">
+        <v>3602</v>
+      </c>
+      <c r="G575" t="n">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B576" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C576" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D576" s="2" t="inlineStr">
+        <is>
+          <t>Jac</t>
+        </is>
+      </c>
+      <c r="E576" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F576" s="2" t="n">
+        <v>2228</v>
+      </c>
+      <c r="G576" s="2" t="n">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B577" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C577" t="n">
+        <v>5</v>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>Jetour</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F577" t="n">
+        <v>1502</v>
+      </c>
+      <c r="G577" t="n">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B578" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C578" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D578" s="2" t="inlineStr">
+        <is>
+          <t>Kia</t>
+        </is>
+      </c>
+      <c r="E578" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F578" s="2" t="n">
+        <v>10241</v>
+      </c>
+      <c r="G578" s="2" t="n">
+        <v>2189</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B579" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C579" t="n">
+        <v>5</v>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>Mazda</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F579" t="n">
+        <v>1457</v>
+      </c>
+      <c r="G579" t="n">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B580" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C580" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D580" s="2" t="inlineStr">
+        <is>
+          <t>Renault</t>
+        </is>
+      </c>
+      <c r="E580" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F580" s="2" t="n">
+        <v>1035</v>
+      </c>
+      <c r="G580" s="2" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B581" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C581" t="n">
+        <v>5</v>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>Sinotruk</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F581" t="n">
+        <v>2086</v>
+      </c>
+      <c r="G581" t="n">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B582" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C582" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D582" s="2" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="E582" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F582" s="2" t="n">
+        <v>1875</v>
+      </c>
+      <c r="G582" s="2" t="n">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B583" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C583" t="n">
+        <v>5</v>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F583" t="n">
+        <v>3044</v>
+      </c>
+      <c r="G583" t="n">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B584" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C584" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D584" s="2" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="E584" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F584" s="2" t="n">
+        <v>1322</v>
+      </c>
+      <c r="G584" s="2" t="n">
+        <v>224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>